<commit_message>
docs: sanitize examples with generic placeholders (no real names)
</commit_message>
<xml_diff>
--- a/example/sample_community_input.xlsx
+++ b/example/sample_community_input.xlsx
@@ -446,81 +446,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Indonesian Cloud Community</t>
+          <t>Example Tech Community</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Komunitas praktisi cloud computing, DevOps, dan arsitektur backend di Jakarta</t>
+          <t>Komunitas praktisi teknologi dan arsitektur cloud di Jakarta</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Faisal Reza</t>
+          <t>PIC Example A</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>faisal@gmail.com</t>
+          <t>pic_a@example.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>08123456789</t>
+          <t>081200000001</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Komunitas Peduli Sampah Jogja</t>
+          <t>Example Green Movement</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gerakan relawan aksi bersih sungai, bank sampah dan daur ulang plastik di Yogyakarta</t>
+          <t>Gerakan relawan bank sampah dan aksi bersih lingkungan di Bandung</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yogi Atmaja</t>
+          <t>PIC Example B</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ogijogjaaa@gmail.com</t>
+          <t>pic_b@example.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>08571234567</t>
+          <t>085700000002</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bandung Runner Club</t>
+          <t>Example Runners Club</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Komunitas lari sehat, marathon enthusiast dan gathering pelari se-Bandung Raya</t>
+          <t>Komunitas lari sehat dan gathering pelari se-Yogyakarta</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Randi Andrian</t>
+          <t>PIC Example C</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>randi@gmail.com</t>
+          <t>pic_c@example.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>081372276161</t>
+          <t>081300000003</t>
         </is>
       </c>
     </row>

</xml_diff>